<commit_message>
Sincronización final de metadatos del Excel antes de cierre de jornada.
</commit_message>
<xml_diff>
--- a/info/Base_Datos_Bendita_2026.xlsx
+++ b/info/Base_Datos_Bendita_2026.xlsx
@@ -1,16 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cesjimp-personal-projects\brands\Bendita\info\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{279C6450-986B-47AA-8C3D-C0B858755E5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Productos" sheetId="1" r:id="rId1"/>
     <sheet name="Combos" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -320,8 +326,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -358,13 +364,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -402,7 +416,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -436,6 +450,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -470,9 +485,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -645,11 +661,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E32"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="128.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -666,7 +687,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -683,7 +704,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -700,7 +721,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -717,7 +738,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -734,7 +755,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -751,7 +772,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -768,7 +789,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -785,7 +806,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -802,7 +823,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -819,7 +840,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -836,7 +857,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -853,7 +874,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -870,7 +891,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -887,7 +908,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -904,7 +925,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -921,7 +942,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -938,7 +959,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -955,7 +976,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -972,7 +993,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -989,7 +1010,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -1006,7 +1027,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>25</v>
       </c>
@@ -1023,7 +1044,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>26</v>
       </c>
@@ -1040,7 +1061,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -1057,7 +1078,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>28</v>
       </c>
@@ -1074,7 +1095,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>29</v>
       </c>
@@ -1091,7 +1112,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>30</v>
       </c>
@@ -1108,7 +1129,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>31</v>
       </c>
@@ -1125,7 +1146,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>32</v>
       </c>
@@ -1142,7 +1163,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>33</v>
       </c>
@@ -1159,7 +1180,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>34</v>
       </c>
@@ -1176,7 +1197,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>35</v>
       </c>
@@ -1199,11 +1220,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1217,7 +1238,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>88</v>
       </c>
@@ -1231,7 +1252,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>89</v>
       </c>
@@ -1245,7 +1266,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>90</v>
       </c>

</xml_diff>